<commit_message>
chore: sync runtime modules and UI/agent updates for github deployment
</commit_message>
<xml_diff>
--- a/example/test_cases_mini.xlsx
+++ b/example/test_cases_mini.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="81">
   <si>
     <t>Category</t>
   </si>
@@ -44,13 +44,13 @@
     <t>NPP VIIRS annual</t>
   </si>
   <si>
-    <t>Retrieve NPP VIIRS annual NTL data for Shanghai from 2015 to 2020.</t>
+    <t>Retrieve NPP VIIRS annual NTL data for Shanghai from 2019 to 2020.</t>
   </si>
   <si>
     <t>DMSP-OLS annual</t>
   </si>
   <si>
-    <t>Retrieve DMSP–OLS annual NTL data for Shanghai from 2005 to 2010.</t>
+    <t>Retrieve DMSP–OLS annual NTL data for Shanghai from 2009 to 2010.</t>
   </si>
   <si>
     <t>NPP-VIIRS-like annual</t>
@@ -218,12 +218,6 @@
   </si>
   <si>
     <t>Calculate NPP-VIIRS average nighttime light intensity (ANTL) in Shanghai each year, from 2015 to 2022, using GEE Python Code,and save it as a csv.</t>
-  </si>
-  <si>
-    <t>Change</t>
-  </si>
-  <si>
-    <t>Download VNP46A2 daily NTL data, and detect the brightness value in the Oriental Pearl Tower, Shanghai before and after the 2024 National Day of China.</t>
   </si>
   <si>
     <t>Thresholded pixel extraction</t>
@@ -1631,7 +1625,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="3"/>
   <cols>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -2064,8 +2058,8 @@
       </c>
     </row>
     <row r="32" ht="15.6" spans="1:4">
-      <c r="A32" s="7">
-        <v>30</v>
+      <c r="A32" s="10">
+        <v>31</v>
       </c>
       <c r="B32" s="10" t="s">
         <v>34</v>
@@ -2078,8 +2072,8 @@
       </c>
     </row>
     <row r="33" ht="15.6" spans="1:4">
-      <c r="A33" s="10">
-        <v>31</v>
+      <c r="A33" s="7">
+        <v>32</v>
       </c>
       <c r="B33" s="10" t="s">
         <v>34</v>
@@ -2092,8 +2086,8 @@
       </c>
     </row>
     <row r="34" ht="15.6" spans="1:4">
-      <c r="A34" s="7">
-        <v>32</v>
+      <c r="A34" s="10">
+        <v>33</v>
       </c>
       <c r="B34" s="10" t="s">
         <v>34</v>
@@ -2106,8 +2100,8 @@
       </c>
     </row>
     <row r="35" ht="15.6" spans="1:4">
-      <c r="A35" s="10">
-        <v>33</v>
+      <c r="A35" s="7">
+        <v>34</v>
       </c>
       <c r="B35" s="10" t="s">
         <v>34</v>
@@ -2119,45 +2113,45 @@
         <v>65</v>
       </c>
     </row>
-    <row r="36" ht="15.6" spans="1:4">
-      <c r="A36" s="7">
+    <row r="36" ht="16.35" spans="1:4">
+      <c r="A36" s="10">
+        <v>35</v>
+      </c>
+      <c r="B36" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="B36" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="C36" s="11" t="s">
+      <c r="C36" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="D36" s="6" t="s">
+      <c r="D36" s="14" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="37" ht="16.35" spans="1:4">
-      <c r="A37" s="10">
-        <v>35</v>
-      </c>
-      <c r="B37" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="C37" s="13" t="s">
+    <row r="37" ht="31.95" spans="1:4">
+      <c r="A37" s="15">
+        <v>36</v>
+      </c>
+      <c r="B37" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="D37" s="14" t="s">
+      <c r="C37" s="15" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="38" ht="31.95" spans="1:4">
-      <c r="A38" s="15">
+      <c r="D37" s="9" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="38" ht="15.6" spans="1:4">
+      <c r="A38" s="16">
         <v>37</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C38" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="D38" s="9" t="s">
+      <c r="D38" s="6" t="s">
         <v>72</v>
       </c>
     </row>
@@ -2165,10 +2159,10 @@
       <c r="A39" s="16">
         <v>38</v>
       </c>
-      <c r="B39" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="C39" s="15" t="s">
+      <c r="B39" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="C39" s="16" t="s">
         <v>73</v>
       </c>
       <c r="D39" s="6" t="s">
@@ -2176,13 +2170,13 @@
       </c>
     </row>
     <row r="40" ht="15.6" spans="1:4">
-      <c r="A40" s="16">
-        <v>36</v>
-      </c>
-      <c r="B40" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="C40" s="16" t="s">
+      <c r="A40" s="15">
+        <v>39</v>
+      </c>
+      <c r="B40" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="C40" s="15" t="s">
         <v>75</v>
       </c>
       <c r="D40" s="6" t="s">
@@ -2190,11 +2184,11 @@
       </c>
     </row>
     <row r="41" ht="15.6" spans="1:4">
-      <c r="A41" s="15">
-        <v>39</v>
+      <c r="A41" s="16">
+        <v>40</v>
       </c>
       <c r="B41" s="15" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C41" s="15" t="s">
         <v>77</v>
@@ -2204,31 +2198,17 @@
       </c>
     </row>
     <row r="42" ht="15.6" spans="1:4">
-      <c r="A42" s="16">
-        <v>40</v>
+      <c r="A42" s="15">
+        <v>41</v>
       </c>
       <c r="B42" s="15" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C42" s="15" t="s">
         <v>79</v>
       </c>
       <c r="D42" s="6" t="s">
         <v>80</v>
-      </c>
-    </row>
-    <row r="43" ht="15.6" spans="1:4">
-      <c r="A43" s="15">
-        <v>41</v>
-      </c>
-      <c r="B43" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="C43" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="D43" s="6" t="s">
-        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>